<commit_message>
Correct expected output in foo_units test script
</commit_message>
<xml_diff>
--- a/conformance_tests/foo_units/test_scripts/TestScript-foo-units.xlsx
+++ b/conformance_tests/foo_units/test_scripts/TestScript-foo-units.xlsx
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="93">
   <si>
     <t xml:space="preserve">Dummy Test</t>
   </si>
@@ -246,31 +246,37 @@
     <t xml:space="preserve">ts_u12</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;=ADD(ts_u1;10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=SUB(ts_u1;10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=MULT(ts_u1;1.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=RAMP(ts_u1; 82; 60; 10)</t>
+    <t xml:space="preserve">=ts_u1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(ts_u1;10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(ts_u1;10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(ts_u1;1.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(ts_u1; 82; 60; 10)</t>
   </si>
   <si>
     <t xml:space="preserve">ts_u13</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;=ADD(ts_y2;100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=SUB(ts_y2;100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=MULT(ts_y2;1.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;=RAMP(ts_y2; 600; 60; 10)</t>
+    <t xml:space="preserve">=ts_y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(ts_y2;100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(ts_y2;100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(ts_y2;1.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(ts_y2; 600; 60; 10)</t>
   </si>
   <si>
     <t xml:space="preserve">Boolean</t>
@@ -418,10 +424,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -565,7 +572,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -776,6 +783,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1043,8 +1054,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="21.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="20.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="21.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="3" width="42.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="3" width="44.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="78" min="12" style="3" width="50.67"/>
@@ -1052,7 +1063,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="1025" style="1" width="9.17"/>
   </cols>
   <sheetData>
-    <row r="1" s="7" customFormat="true" ht="16.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="7" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1095,7 +1106,7 @@
       <c r="BP1" s="8"/>
       <c r="BQ1" s="9"/>
     </row>
-    <row r="2" s="10" customFormat="true" ht="16.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="10" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1123,7 +1134,7 @@
       <c r="BP2" s="11"/>
       <c r="BQ2" s="12"/>
     </row>
-    <row r="3" s="10" customFormat="true" ht="16.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="10" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1211,7 +1222,7 @@
       <c r="BY3" s="5"/>
       <c r="BZ3" s="5"/>
     </row>
-    <row r="4" s="10" customFormat="true" ht="16.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" s="10" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
@@ -1232,7 +1243,7 @@
       <c r="BP4" s="11"/>
       <c r="BQ4" s="12"/>
     </row>
-    <row r="5" s="10" customFormat="true" ht="16.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="10" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
@@ -2576,21 +2587,20 @@
       <c r="F19" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G19" s="35" t="e">
-        <f aca="false">ts_u1</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="H19" s="35" t="s">
+      <c r="G19" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="I19" s="35" t="s">
+      <c r="H19" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="J19" s="35" t="s">
+      <c r="I19" s="39" t="s">
         <v>37</v>
       </c>
+      <c r="J19" s="39" t="s">
+        <v>38</v>
+      </c>
       <c r="K19" s="39" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L19" s="36"/>
       <c r="M19" s="36"/>
@@ -2665,7 +2675,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="34" t="n">
@@ -2677,21 +2687,20 @@
       <c r="F20" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="G20" s="35" t="e">
-        <f aca="false">ts_y2</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="H20" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="I20" s="35" t="s">
+      <c r="G20" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="J20" s="35" t="s">
+      <c r="H20" s="39" t="s">
         <v>42</v>
       </c>
+      <c r="I20" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="J20" s="39" t="s">
+        <v>44</v>
+      </c>
       <c r="K20" s="39" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
@@ -2763,35 +2772,35 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C21" s="33"/>
       <c r="D21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K21" s="34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
@@ -2863,35 +2872,35 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B22" s="32" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C22" s="33"/>
       <c r="D22" s="34" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K22" s="34" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
@@ -2963,35 +2972,35 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C23" s="33"/>
       <c r="D23" s="34" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
@@ -3063,35 +3072,35 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B24" s="32" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C24" s="33"/>
       <c r="D24" s="34" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K24" s="34" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
@@ -3163,35 +3172,35 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C25" s="33"/>
       <c r="D25" s="40" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K25" s="34" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
@@ -3263,35 +3272,35 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B26" s="32" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C26" s="33"/>
       <c r="D26" s="34" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="K26" s="34" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
@@ -3363,35 +3372,35 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C27" s="33"/>
       <c r="D27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L27" s="36"/>
       <c r="M27" s="36"/>
@@ -3543,10 +3552,10 @@
     </row>
     <row r="29" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="41" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B29" s="41" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="42"/>
@@ -3563,35 +3572,35 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B30" s="32" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" s="33"/>
       <c r="D30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J30" s="40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K30" s="40" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L30" s="46"/>
       <c r="M30" s="46"/>
@@ -3666,13 +3675,13 @@
         <v>11</v>
       </c>
       <c r="B31" s="49" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C31" s="50"/>
       <c r="D31" s="40"/>
       <c r="E31" s="40"/>
       <c r="F31" s="51" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G31" s="36"/>
       <c r="H31" s="36"/>
@@ -3749,10 +3758,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="49" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B32" s="49" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C32" s="50"/>
       <c r="D32" s="40"/>
@@ -3835,13 +3844,13 @@
     </row>
     <row r="33" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="41" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B33" s="41" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D33" s="42"/>
       <c r="E33" s="42"/>
@@ -3860,13 +3869,13 @@
         <v>17</v>
       </c>
       <c r="B34" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" s="50" t="n">
-        <v>0</v>
+        <v>74</v>
+      </c>
+      <c r="C34" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D34" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E34" s="34" t="n">
         <v>70</v>
@@ -3962,13 +3971,13 @@
         <v>19</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="C35" s="50" t="n">
-        <v>0</v>
+        <v>81</v>
+      </c>
+      <c r="C35" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D35" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E35" s="34" t="n">
         <v>500</v>
@@ -4064,13 +4073,13 @@
         <v>21</v>
       </c>
       <c r="B36" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" s="53" t="n">
+        <v>1E-006</v>
+      </c>
+      <c r="D36" s="40" t="s">
         <v>80</v>
-      </c>
-      <c r="C36" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="40" t="s">
-        <v>78</v>
       </c>
       <c r="E36" s="34" t="n">
         <v>800</v>
@@ -4166,13 +4175,13 @@
         <v>23</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C37" s="50" t="n">
-        <v>0</v>
+        <v>83</v>
+      </c>
+      <c r="C37" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D37" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E37" s="34" t="n">
         <v>60</v>
@@ -4268,13 +4277,13 @@
         <v>25</v>
       </c>
       <c r="B38" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="C38" s="50" t="n">
-        <v>0</v>
+        <v>84</v>
+      </c>
+      <c r="C38" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D38" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E38" s="34" t="n">
         <v>200</v>
@@ -4370,13 +4379,13 @@
         <v>17</v>
       </c>
       <c r="B39" s="32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C39" s="50" t="n">
         <v>0.5</v>
       </c>
       <c r="D39" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E39" s="34" t="n">
         <v>70</v>
@@ -4472,13 +4481,13 @@
         <v>19</v>
       </c>
       <c r="B40" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C40" s="50" t="n">
         <v>5</v>
       </c>
       <c r="D40" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E40" s="34" t="n">
         <v>500</v>
@@ -4574,13 +4583,13 @@
         <v>21</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C41" s="50" t="n">
         <v>5</v>
       </c>
       <c r="D41" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E41" s="34" t="n">
         <v>800</v>
@@ -4676,13 +4685,13 @@
         <v>23</v>
       </c>
       <c r="B42" s="32" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C42" s="50" t="n">
         <v>5</v>
       </c>
       <c r="D42" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E42" s="34" t="n">
         <v>60</v>
@@ -4778,13 +4787,13 @@
         <v>25</v>
       </c>
       <c r="B43" s="32" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C43" s="50" t="n">
         <v>5</v>
       </c>
       <c r="D43" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E43" s="34" t="n">
         <v>200</v>
@@ -4880,13 +4889,13 @@
         <v>32</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C44" s="50" t="n">
         <v>0.1</v>
       </c>
       <c r="D44" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E44" s="36" t="n">
         <v>4</v>
@@ -4982,13 +4991,13 @@
         <v>17</v>
       </c>
       <c r="B45" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="C45" s="50" t="n">
-        <v>0</v>
+        <v>91</v>
+      </c>
+      <c r="C45" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D45" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E45" s="34" t="n">
         <v>70</v>
@@ -5006,7 +5015,7 @@
         <v>64</v>
       </c>
       <c r="J45" s="35" t="n">
-        <v>84.4</v>
+        <v>81.4</v>
       </c>
       <c r="K45" s="35" t="n">
         <v>82</v>
@@ -5017,13 +5026,13 @@
         <v>19</v>
       </c>
       <c r="B46" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="C46" s="50" t="n">
-        <v>0</v>
+        <v>92</v>
+      </c>
+      <c r="C46" s="53" t="n">
+        <v>1E-006</v>
       </c>
       <c r="D46" s="40" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E46" s="34" t="n">
         <v>500</v>
@@ -5050,7 +5059,7 @@
   </sheetData>
   <conditionalFormatting sqref="M34:ZY44 L8:ZY27 G28:ZY28 L34:L38 L41:L44">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>#ref!&lt;&gt;G8</formula>
+      <formula>#ref!&lt;&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>